<commit_message>
Week 40: replace interest export with corrected HubSpot data (120 partners) and update analysis, charts, slides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkDZ43fAxsiGHwtPuUQvfi
</commit_message>
<xml_diff>
--- a/challenge-ia/semaines/2026-S40/export-hubspot-opportunites-ia-2026-10-01.xlsx
+++ b/challenge-ia/semaines/2026-S40/export-hubspot-opportunites-ia-2026-10-01.xlsx
@@ -99,11 +99,11 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Jennifer Pereira</t>
+          <t>Corinne BAROUKH</t>
         </is>
       </c>
     </row>
@@ -118,7 +118,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Alain Babaci</t>
+          <t>vincent Del Campo</t>
         </is>
       </c>
     </row>
@@ -129,11 +129,11 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Corinne BAROUKH</t>
+          <t>Alain Babaci</t>
         </is>
       </c>
     </row>
@@ -144,11 +144,11 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>vincent Del Campo</t>
+          <t>Jennifer Pereira</t>
         </is>
       </c>
     </row>
@@ -163,7 +163,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Corinne BAROUKH</t>
+          <t>Alain Babaci</t>
         </is>
       </c>
     </row>
@@ -178,7 +178,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Alain Babaci</t>
+          <t>Corinne BAROUKH</t>
         </is>
       </c>
     </row>
@@ -249,16 +249,16 @@
         </is>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46311.70233184028</v>
+        <v>46353.45272105324</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>521464810741</t>
+          <t>521452546241</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>8368197845</t>
+          <t>448730881217</t>
         </is>
       </c>
     </row>
@@ -309,16 +309,16 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46355.48854571759</v>
+        <v>46355.489418854166</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>518714945748</t>
+          <t>518874716376</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>7877376458</t>
+          <t>7824673476</t>
         </is>
       </c>
     </row>
@@ -360,25 +360,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jennifer Pereira</t>
+          <t>Corinne BAROUKH</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dstny UCaaS; Dstny Digital Assistant</t>
+          <t>Dstny Digital Assistant</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46326.41874197916</v>
+        <v>46311.70233184028</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>495031382265</t>
+          <t>521464810741</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>7650923966</t>
+          <t>8368197845</t>
         </is>
       </c>
     </row>
@@ -390,7 +390,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Corinne BAROUKH</t>
+          <t>Jennifer Pereira</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -399,16 +399,16 @@
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46353.45272105324</v>
+        <v>46355.48854571759</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>521452546241</t>
+          <t>518714945748</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>448730881217</t>
+          <t>7877376458</t>
         </is>
       </c>
     </row>
@@ -420,7 +420,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Corinne BAROUKH</t>
+          <t>Alain Babaci</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -429,16 +429,16 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>46326.642579039355</v>
+        <v>46325.79478199074</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>519652009200</t>
+          <t>511203980475</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>7873964994</t>
+          <t>10061742314</t>
         </is>
       </c>
     </row>
@@ -455,20 +455,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dstny Digital Assistant</t>
+          <t>Dstny UCaaS; Dstny Digital Assistant</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>46355.489418854166</v>
+        <v>46326.41874197916</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>518874716376</t>
+          <t>495031382265</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>7824673476</t>
+          <t>7650923966</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alain Babaci</t>
+          <t>Corinne BAROUKH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -489,16 +489,16 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>46325.79478199074</v>
+        <v>46326.642579039355</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>511203980475</t>
+          <t>519652009200</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10061742314</t>
+          <t>7873964994</t>
         </is>
       </c>
     </row>
@@ -510,25 +510,25 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Corinne BAROUKH</t>
+          <t>Alain Babaci</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dstny Digital Assistant</t>
+          <t>Dstny Digital Assistant; VoIPcube</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>46325.44813873843</v>
+        <v>46325.79465079861</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>521687658744</t>
+          <t>511360288968</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>8367713474</t>
+          <t>10061742314</t>
         </is>
       </c>
     </row>
@@ -540,25 +540,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alain Babaci</t>
+          <t>Corinne BAROUKH</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dstny Digital Assistant; VoIPcube</t>
+          <t>Dstny Digital Assistant</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>46325.79465079861</v>
+        <v>46325.44813873843</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>511360288968</t>
+          <t>521687658744</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10061742314</t>
+          <t>8367713474</t>
         </is>
       </c>
     </row>

</xml_diff>